<commit_message>
Complete Smart Multi-Face Attendance System with Web Dashboard
</commit_message>
<xml_diff>
--- a/attendance_log.xlsx
+++ b/attendance_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -966,6 +966,94 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>joel</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>12:38:00</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>joel</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>13:43:26</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>joel</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>13:44:03</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>joel</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>14:13:34</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>